<commit_message>
Update Table S1 - Bulk RNASeq STAR mapping and FeatureCounts Quantification.xlsx
</commit_message>
<xml_diff>
--- a/Directory S1 - Bulk/Table S1 - Bulk RNASeq STAR mapping and FeatureCounts Quantification.xlsx
+++ b/Directory S1 - Bulk/Table S1 - Bulk RNASeq STAR mapping and FeatureCounts Quantification.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/johnbriseno/Desktop/Manuscripts/Ch2_Bulk_Atlas/Supplemental/Bulk Supp./"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/johnbriseno/Desktop/Manuscripts/Ch2_Bulk_Atlas/Supplemental/GitHubRepo/Directory S1 - Bulk/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AECE4E4A-D588-884F-9D48-DCBC29941771}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB46726D-1EAB-0944-9976-5214A900B202}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="10540" yWindow="760" windowWidth="23940" windowHeight="21580" xr2:uid="{A5420101-CBE5-AC45-86CD-BAFE927FB4D4}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="163" uniqueCount="126">
   <si>
     <t>MS4_WBL_167730</t>
   </si>
@@ -405,6 +405,15 @@
   </si>
   <si>
     <t>FS9_OVRY_190965</t>
+  </si>
+  <si>
+    <t>https://www.ncbi.nlm.nih.gov/biosample/SAMN64208675</t>
+  </si>
+  <si>
+    <t>https://www.ncbi.nlm.nih.gov/biosample/?term=SAMN64208709</t>
+  </si>
+  <si>
+    <t>https://www.ncbi.nlm.nih.gov/biosample/?term=SAMN64208755</t>
   </si>
 </sst>
 </file>
@@ -881,6 +890,9 @@
       <c r="B2" s="1" t="s">
         <v>55</v>
       </c>
+      <c r="C2" s="7" t="s">
+        <v>123</v>
+      </c>
       <c r="D2" s="8">
         <v>33455192</v>
       </c>
@@ -1016,6 +1028,9 @@
       <c r="B8" s="1" t="s">
         <v>56</v>
       </c>
+      <c r="C8" s="7" t="s">
+        <v>124</v>
+      </c>
       <c r="D8" s="8">
         <v>41759128</v>
       </c>
@@ -1035,6 +1050,9 @@
       </c>
       <c r="B9" s="1" t="s">
         <v>56</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>125</v>
       </c>
       <c r="D9" s="8">
         <v>33218470</v>
@@ -2156,6 +2174,9 @@
     <hyperlink ref="C35" r:id="rId47" xr:uid="{5E516D3B-5E0C-4746-A84F-28BF69B43AAF}"/>
     <hyperlink ref="C37" r:id="rId48" xr:uid="{8273F768-C633-8847-928A-EB0226AE5ADE}"/>
     <hyperlink ref="C38" r:id="rId49" xr:uid="{A9F41C10-4F9E-1F45-83EC-FC2B917AE4BE}"/>
+    <hyperlink ref="C2" r:id="rId50" xr:uid="{EE24185C-D43F-BD4B-9457-BDCD99434C26}"/>
+    <hyperlink ref="C8" r:id="rId51" xr:uid="{2BF048D8-5032-CB4D-B7CD-1F5738588DE1}"/>
+    <hyperlink ref="C9" r:id="rId52" xr:uid="{4BD39ADD-4C67-8D4B-BE87-CFED46EB0395}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>